<commit_message>
Add SOH report for 2026-10-27
</commit_message>
<xml_diff>
--- a/reports/SOH_27_10_2026.xlsx
+++ b/reports/SOH_27_10_2026.xlsx
@@ -1478,7 +1478,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>10939</v>
+        <v>10915</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>10251</v>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>9408</v>
@@ -2374,7 +2374,7 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>750</v>
+        <v>738</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>10487</v>
@@ -2402,7 +2402,7 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>1134</v>
+        <v>1122</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>8018</v>
@@ -3298,7 +3298,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>14752</v>
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="E165" s="3" t="n">
         <v>14115</v>
@@ -10082,7 +10082,7 @@
         </is>
       </c>
       <c r="D348" s="2" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E348" s="3" t="n">
         <v>4000</v>
@@ -10334,7 +10334,7 @@
         </is>
       </c>
       <c r="D357" s="2" t="n">
-        <v>536</v>
+        <v>524</v>
       </c>
       <c r="E357" s="3" t="n">
         <v>8597</v>
@@ -10362,7 +10362,7 @@
         </is>
       </c>
       <c r="D358" s="2" t="n">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="E358" s="3" t="n">
         <v>8597</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="D359" s="2" t="n">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="E359" s="3" t="n">
         <v>8597</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="D363" s="2" t="n">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="E363" s="3" t="n">
         <v>4708</v>
@@ -10530,7 +10530,7 @@
         </is>
       </c>
       <c r="D364" s="2" t="n">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="E364" s="3" t="n">
         <v>4708</v>
@@ -10558,7 +10558,7 @@
         </is>
       </c>
       <c r="D365" s="2" t="n">
-        <v>795</v>
+        <v>723</v>
       </c>
       <c r="E365" s="3" t="n">
         <v>12500</v>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="D373" s="2" t="n">
-        <v>1413</v>
+        <v>1329</v>
       </c>
       <c r="E373" s="3" t="n">
         <v>40000</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="D375" s="2" t="n">
-        <v>909</v>
+        <v>861</v>
       </c>
       <c r="E375" s="3" t="n">
         <v>40000</v>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D377" s="2" t="n">
-        <v>852</v>
+        <v>786</v>
       </c>
       <c r="E377" s="3" t="n">
         <v>40000</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="D379" s="2" t="n">
-        <v>464</v>
+        <v>392</v>
       </c>
       <c r="E379" s="3" t="n">
         <v>40000</v>
@@ -11286,7 +11286,7 @@
         </is>
       </c>
       <c r="D391" s="2" t="n">
-        <v>669</v>
+        <v>654</v>
       </c>
       <c r="E391" s="3" t="n">
         <v>51000</v>
@@ -11342,7 +11342,7 @@
         </is>
       </c>
       <c r="D393" s="2" t="n">
-        <v>1031</v>
+        <v>991</v>
       </c>
       <c r="E393" s="3" t="n">
         <v>51000</v>
@@ -11398,7 +11398,7 @@
         </is>
       </c>
       <c r="D395" s="2" t="n">
-        <v>1337</v>
+        <v>1320</v>
       </c>
       <c r="E395" s="3" t="n">
         <v>51000</v>
@@ -11454,7 +11454,7 @@
         </is>
       </c>
       <c r="D397" s="2" t="n">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="E397" s="3" t="n">
         <v>51000</v>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="D399" s="2" t="n">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E399" s="3" t="n">
         <v>51000</v>
@@ -12126,7 +12126,7 @@
         </is>
       </c>
       <c r="D421" s="2" t="n">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="E421" s="3" t="n">
         <v>21000</v>
@@ -12182,7 +12182,7 @@
         </is>
       </c>
       <c r="D423" s="2" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="E423" s="3" t="n">
         <v>21000</v>
@@ -12238,7 +12238,7 @@
         </is>
       </c>
       <c r="D425" s="2" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E425" s="3" t="n">
         <v>21000</v>
@@ -12434,7 +12434,7 @@
         </is>
       </c>
       <c r="D432" s="2" t="n">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="E432" s="3" t="n">
         <v>2500</v>
@@ -12546,7 +12546,7 @@
         </is>
       </c>
       <c r="D436" s="2" t="n">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="E436" s="3" t="n">
         <v>3500</v>
@@ -12826,7 +12826,7 @@
         </is>
       </c>
       <c r="D446" s="2" t="n">
-        <v>4588</v>
+        <v>4563</v>
       </c>
       <c r="E446" s="3" t="n">
         <v>2500</v>
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="D505" s="2" t="n">
-        <v>861</v>
+        <v>849</v>
       </c>
       <c r="E505" s="3" t="n">
         <v>7564</v>
@@ -15850,7 +15850,7 @@
         </is>
       </c>
       <c r="D554" s="2" t="n">
-        <v>1316</v>
+        <v>1306</v>
       </c>
       <c r="E554" s="3" t="n">
         <v>11078</v>
@@ -17866,7 +17866,7 @@
         </is>
       </c>
       <c r="D626" s="2" t="n">
-        <v>750</v>
+        <v>726</v>
       </c>
       <c r="E626" s="3" t="n">
         <v>8626</v>

</xml_diff>